<commit_message>
2026, rättningar uppdatering 1
2026, rättningar uppdatering 1
</commit_message>
<xml_diff>
--- a/Bibsam_tidskriftslistor/Uppdateringar/Tidskriftslistor_ändringar_2026.xlsx
+++ b/Bibsam_tidskriftslistor/Uppdateringar/Tidskriftslistor_ändringar_2026.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\larher\Documents\GitHub\oa-tskr\Bibsam_tidskriftslistor\Uppdateringar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{53F5BB8E-EC0D-4C7D-924C-93120E3BC0FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{595DEB9B-B058-4A68-9813-D30C73D92CB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nr1_Jan13" sheetId="1" r:id="rId1"/>
     <sheet name="Nr2_Jan19" sheetId="2" r:id="rId2"/>
+    <sheet name="Nr3_Jan20" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3666" uniqueCount="1702">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3688" uniqueCount="1709">
   <si>
     <t>Imprint</t>
   </si>
@@ -5132,6 +5133,27 @@
   </si>
   <si>
     <t>dubblett borttagen</t>
+  </si>
+  <si>
+    <t>2631-4940</t>
+  </si>
+  <si>
+    <t>BMJ Surgery, Interventions, &amp; Health Technologies</t>
+  </si>
+  <si>
+    <t>https://sit.bmj.com/</t>
+  </si>
+  <si>
+    <t>2978-1809</t>
+  </si>
+  <si>
+    <t>BMJ Connections Surgery</t>
+  </si>
+  <si>
+    <t>https://connectionssurgery.bmj.com/</t>
+  </si>
+  <si>
+    <t>ny</t>
   </si>
 </sst>
 </file>
@@ -17466,4 +17488,86 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A182B91-835E-4E83-B5C7-A60B1DA82CFC}">
+  <dimension ref="A1:H3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>307</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1702</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1703</v>
+      </c>
+      <c r="E2" t="s">
+        <v>1704</v>
+      </c>
+      <c r="F2" t="s">
+        <v>18</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>307</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1705</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1706</v>
+      </c>
+      <c r="E3" t="s">
+        <v>1707</v>
+      </c>
+      <c r="F3" t="s">
+        <v>18</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>1708</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Rättningar till uppdatering 6
Rättningar till uppdatering 6
</commit_message>
<xml_diff>
--- a/Bibsam_tidskriftslistor/Uppdateringar/Tidskriftslistor_ändringar_2026.xlsx
+++ b/Bibsam_tidskriftslistor/Uppdateringar/Tidskriftslistor_ändringar_2026.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\larher\Documents\GitHub\oa-tskr\Bibsam_tidskriftslistor\Uppdateringar\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8390B5B8-6AD7-4A7A-B970-F760DFC5B974}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB0450E6-DFDA-4318-A895-5A9EB0430ECC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nr1_Jan13" sheetId="1" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <sheet name="Nr4_Mars6" sheetId="5" r:id="rId5"/>
     <sheet name="Nr5_Mars16" sheetId="6" r:id="rId6"/>
     <sheet name="Nr6_April13" sheetId="7" r:id="rId7"/>
+    <sheet name="Rättningar_April16" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -31,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5464" uniqueCount="2354">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5493" uniqueCount="2355">
   <si>
     <t>Imprint</t>
   </si>
@@ -7093,6 +7094,9 @@
   </si>
   <si>
     <t>https://publicera.kb.se/ejpae</t>
+  </si>
+  <si>
+    <t>Tar bort, blev felaktigt tillagd i uppdatering 6</t>
   </si>
 </sst>
 </file>
@@ -25457,4 +25461,109 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16C4AC14-6653-464E-95B3-5FC270042EE8}">
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2309</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2310</v>
+      </c>
+      <c r="E2" t="s">
+        <v>2311</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2321</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2322</v>
+      </c>
+      <c r="E3" t="s">
+        <v>2323</v>
+      </c>
+      <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H3" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>2308</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2315</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2316</v>
+      </c>
+      <c r="E4" t="s">
+        <v>2317</v>
+      </c>
+      <c r="F4" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" t="s">
+        <v>2354</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>